<commit_message>
Actualización: Parámetros de impresión
</commit_message>
<xml_diff>
--- a/Parámetros de impresión.xlsx
+++ b/Parámetros de impresión.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arena\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD79A29B-CE25-44A1-9CC1-61180A1F363B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A37632C-B34E-4D95-9E8C-448225D17055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F46B5450-57FD-4274-88ED-D57A14AACDFF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="14">
   <si>
     <t>Fecha</t>
   </si>
@@ -128,12 +128,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -473,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A404F36C-DD92-42BB-A7E5-A4FC7F6D61B9}">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="16.88671875" customWidth="1"/>
@@ -1779,6 +1785,66 @@
         <v>6</v>
       </c>
     </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="2">
+        <v>46073</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D66" s="4">
+        <v>20</v>
+      </c>
+      <c r="E66" s="5">
+        <v>40</v>
+      </c>
+      <c r="F66" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="2">
+        <v>46073</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="4">
+        <v>20</v>
+      </c>
+      <c r="E67" s="5">
+        <v>40</v>
+      </c>
+      <c r="F67" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="2">
+        <v>46073</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="4">
+        <v>18</v>
+      </c>
+      <c r="E68" s="5">
+        <v>36</v>
+      </c>
+      <c r="F68" s="5">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actuaoización 2.0 datos impresión
</commit_message>
<xml_diff>
--- a/Parámetros de impresión.xlsx
+++ b/Parámetros de impresión.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arena\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A37632C-B34E-4D95-9E8C-448225D17055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{084FCF10-6542-4FA5-93BB-40BFE5D37E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F46B5450-57FD-4274-88ED-D57A14AACDFF}"/>
   </bookViews>
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -137,12 +137,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1795,13 +1789,13 @@
       <c r="C66" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D66" s="4">
+      <c r="D66" s="1">
         <v>20</v>
       </c>
-      <c r="E66" s="5">
+      <c r="E66" s="3">
         <v>40</v>
       </c>
-      <c r="F66" s="5">
+      <c r="F66" s="3">
         <v>6</v>
       </c>
     </row>
@@ -1815,13 +1809,13 @@
       <c r="C67" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D67" s="4">
+      <c r="D67" s="1">
         <v>20</v>
       </c>
-      <c r="E67" s="5">
+      <c r="E67" s="3">
         <v>40</v>
       </c>
-      <c r="F67" s="5">
+      <c r="F67" s="3">
         <v>7</v>
       </c>
     </row>
@@ -1835,13 +1829,13 @@
       <c r="C68" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D68" s="4">
-        <v>18</v>
-      </c>
-      <c r="E68" s="5">
+      <c r="D68" s="1">
+        <v>18</v>
+      </c>
+      <c r="E68" s="3">
         <v>36</v>
       </c>
-      <c r="F68" s="5">
+      <c r="F68" s="3">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adición imágenes viabilidad celular
</commit_message>
<xml_diff>
--- a/Parámetros de impresión.xlsx
+++ b/Parámetros de impresión.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arena\Desktop\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{084FCF10-6542-4FA5-93BB-40BFE5D37E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F4376D-4305-4A77-8934-2E0BEE5DF890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F46B5450-57FD-4274-88ED-D57A14AACDFF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="14">
   <si>
     <t>Fecha</t>
   </si>
@@ -473,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A404F36C-DD92-42BB-A7E5-A4FC7F6D61B9}">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="16.88671875" customWidth="1"/>
@@ -1779,66 +1779,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="2">
-        <v>46073</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D66" s="1">
-        <v>20</v>
-      </c>
-      <c r="E66" s="3">
-        <v>40</v>
-      </c>
-      <c r="F66" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="2">
-        <v>46073</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" s="1">
-        <v>20</v>
-      </c>
-      <c r="E67" s="3">
-        <v>40</v>
-      </c>
-      <c r="F67" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="2">
-        <v>46073</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D68" s="1">
-        <v>18</v>
-      </c>
-      <c r="E68" s="3">
-        <v>36</v>
-      </c>
-      <c r="F68" s="3">
-        <v>6</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>